<commit_message>
Improve assistant chat experience
</commit_message>
<xml_diff>
--- a/outputs/tppc_lims_master/TPPC_Instruments_final.xlsx
+++ b/outputs/tppc_lims_master/TPPC_Instruments_final.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instruments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="QA_Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1736,7 +1736,11 @@
           <t>آنالایزر گوگرد XRF</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>آنالایزر گوگرد XRF</t>
+        </is>
+      </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
           <t>EDXRF Sulfur Analyzer</t>
@@ -2491,7 +2495,11 @@
           <t>دستگاه رنگ سیبولت</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>رنگ‌سنج سیبولت</t>
+        </is>
+      </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Saybolt Colorimeter</t>

</xml_diff>